<commit_message>
Add Phase 2 Direct Expense: DE cost element and per-contract aggregation
- 31_direct_expense.xlsx: new test fixture (WO-attributed, contract-attributed,
  negative reversal, zero-amount, and unassigned-WO rows)
- 04_cost_element.xlsx: add DE (직접경비, is_manufacturing=Y)
- calculate_actual_direct_expense_by_contract(): rolls WO-attributed expenses up
  through work_order.contract_no and contract-attributed ones directly; the
  31_direct_expense.xlsx amount is the sole canonical source and GL amounts are
  never re-aggregated
- validate_direct_expense(): reuses duplicate_keys()/UNKNOWN_CONTRACT/UNKNOWN_WO/
  INVALID_DECIMAL and adds one new code, EXPENSE_TARGET_CONFLICT, for rows
  carrying both wo_no and contract_no
- GL account 53900 is deliberately left unmapped, so the existing UNMAPPED_GL
  (E-012) scenario is preserved
- No DM/DL/OH/GA calculation logic modified
</commit_message>
<xml_diff>
--- a/hanbit_mvp_dataset_phase1/04_cost_element.xlsx
+++ b/hanbit_mvp_dataset_phase1/04_cost_element.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cost_element" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="cost_element" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'cost_element'!$A$1:$C$5</definedName>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,6 +509,23 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>직접경비</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>

</xml_diff>